<commit_message>
Update test data and CI configuration
</commit_message>
<xml_diff>
--- a/testdata/userdata.xlsx
+++ b/testdata/userdata.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\python\notes-api\OrangeHrm\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C35AF369-2556-4406-9806-D75A9673C1ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B64A5707-9EBA-4FB8-9C31-2E0CB9478C91}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -74,22 +74,22 @@
     <t>empname</t>
   </si>
   <si>
-    <t>rerqt@123</t>
-  </si>
-  <si>
-    <t>fk3244432</t>
-  </si>
-  <si>
-    <t>jkxA12352</t>
-  </si>
-  <si>
-    <t>ledlst@1262</t>
-  </si>
-  <si>
-    <t>n</t>
-  </si>
-  <si>
-    <t>m</t>
+    <t>t</t>
+  </si>
+  <si>
+    <t>j</t>
+  </si>
+  <si>
+    <t>fkj233</t>
+  </si>
+  <si>
+    <t>jdef234</t>
+  </si>
+  <si>
+    <t>rerqt@4566</t>
+  </si>
+  <si>
+    <t>ledlst@656</t>
   </si>
 </sst>
 </file>
@@ -448,16 +448,16 @@
         <v>4</v>
       </c>
       <c r="B2" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="C2" t="s">
         <v>5</v>
       </c>
       <c r="D2" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
@@ -465,16 +465,16 @@
         <v>4</v>
       </c>
       <c r="B3" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="C3" t="s">
         <v>5</v>
       </c>
       <c r="D3" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
stabilze the creation tests
</commit_message>
<xml_diff>
--- a/testdata/userdata.xlsx
+++ b/testdata/userdata.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\python\notes-api\OrangeHrm\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8C9CC34-6C35-4CE2-A4ED-40DC277EFA0C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{102C0849-8273-4A1C-915C-94A3171D839F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -74,9 +74,6 @@
     <t>empname</t>
   </si>
   <si>
-    <t>g</t>
-  </si>
-  <si>
     <t>k</t>
   </si>
   <si>
@@ -90,6 +87,9 @@
   </si>
   <si>
     <t>ledlst@6563</t>
+  </si>
+  <si>
+    <t>d</t>
   </si>
 </sst>
 </file>
@@ -448,16 +448,16 @@
         <v>4</v>
       </c>
       <c r="B2" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="C2" t="s">
         <v>5</v>
       </c>
       <c r="D2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
@@ -465,16 +465,16 @@
         <v>4</v>
       </c>
       <c r="B3" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C3" t="s">
         <v>5</v>
       </c>
       <c r="D3" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
   </sheetData>

</xml_diff>